<commit_message>
Deploying to gh-pages from @ samply/cce-fhir-ig@8bcefe49bbc5f4b8fe5614a79dd24cd925fafd37 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-DiagnosticConfirmationCS.xlsx
+++ b/CodeSystem-DiagnosticConfirmationCS.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.5.0</t>
+    <t>0.6.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-18T08:48:21+00:00</t>
+    <t>2026-09-18T09:32:10+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ samply/cce-fhir-ig@d41a0b7c5426a72984263afe11c663b442913305 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-DiagnosticConfirmationCS.xlsx
+++ b/CodeSystem-DiagnosticConfirmationCS.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.6.0</t>
+    <t>0.6.1</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-18T09:32:10+00:00</t>
+    <t>2026-09-18T11:05:59+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ samply/cce-fhir-ig@7bbc946fbf51b43b99183ada6f0cfc09d2ac8167 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-DiagnosticConfirmationCS.xlsx
+++ b/CodeSystem-DiagnosticConfirmationCS.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.6.1</t>
+    <t>0.6.2</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-18T14:51:59+00:00</t>
+    <t>2026-09-21T07:38:15+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ samply/cce-fhir-ig@c4ee1af4d186efacc06cdd2e9239ca3ffbde03b4 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-DiagnosticConfirmationCS.xlsx
+++ b/CodeSystem-DiagnosticConfirmationCS.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.6.2</t>
+    <t>0.6.3</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-21T09:00:44+00:00</t>
+    <t>2026-09-21T09:40:01+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ samply/cce-fhir-ig@ed59293102f4d641af1db7c4675f07ffe76013f7 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-DiagnosticConfirmationCS.xlsx
+++ b/CodeSystem-DiagnosticConfirmationCS.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.6.3</t>
+    <t>0.6.4</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-23T11:26:04+00:00</t>
+    <t>2026-10-22T11:42:36+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>